<commit_message>
refactor(api/malla): extract agrupación resolution logic for optatives
Extract duplicated agrupación lookup and template-based creation logic into a private `resolveAgrupacionDestino` helper method, used by both `asignarOptativaAgrupacion` and `asignarOptativasBatch` endpoints. Remove the `exists:agrupaciones,ID_Agrupacion` validation rule to support passing predefined plantilla IDs, add explicit 422 error handling for invalid target agrupaciones, and update all database operations to use the resolved real agrupacion instance. This reduces code duplication, improves readability and maintainability, and enables creating agrupaciones from plantillas when assigning optatives to a curricular malla.
</commit_message>
<xml_diff>
--- a/files_tests/FORMATO DE CARGA - OPTATIVA.xlsx
+++ b/files_tests/FORMATO DE CARGA - OPTATIVA.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="228">
   <si>
     <t>PROGRAMA CURRICULAR</t>
   </si>
@@ -817,7 +817,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -877,9 +877,6 @@
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
@@ -1340,10 +1337,18 @@
       <c r="C5" s="12">
         <v>4.0</v>
       </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
+      <c r="D5" s="11">
+        <v>4101210.0</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="H5" s="8">
         <v>4200686.0</v>
       </c>
@@ -1432,10 +1437,18 @@
       <c r="C7" s="12">
         <v>4.0</v>
       </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
+      <c r="D7" s="11">
+        <v>4101553.0</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="H7" s="8">
         <v>4200686.0</v>
       </c>
@@ -1624,10 +1637,18 @@
       <c r="C11" s="12">
         <v>13.0</v>
       </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
+      <c r="D11" s="11">
+        <v>4201082.0</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="H11" s="8">
         <v>4201064.0</v>
       </c>
@@ -2066,6 +2087,18 @@
       <c r="C20" s="11">
         <v>25.0</v>
       </c>
+      <c r="D20" s="11">
+        <v>4101392.0</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="H20" s="8">
         <v>4100552.0</v>
       </c>
@@ -2352,7 +2385,19 @@
       <c r="C26" s="11">
         <v>25.0</v>
       </c>
-      <c r="H26" s="20">
+      <c r="D26" s="11">
+        <v>4100566.0</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F26" s="11">
+        <v>3.0</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H26" s="8">
         <v>4100538.0</v>
       </c>
       <c r="I26" s="11" t="s">
@@ -2361,7 +2406,7 @@
       <c r="J26" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="K26" s="21"/>
+      <c r="K26" s="20"/>
       <c r="L26" s="10"/>
       <c r="M26" s="10"/>
       <c r="N26" s="10"/>
@@ -2730,6 +2775,18 @@
       <c r="C34" s="11">
         <v>37.0</v>
       </c>
+      <c r="D34" s="11">
+        <v>4100638.0</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F34" s="11">
+        <v>4.0</v>
+      </c>
+      <c r="G34" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="H34" s="11">
         <v>4100637.0</v>
       </c>
@@ -2818,6 +2875,18 @@
       <c r="C36" s="11">
         <v>40.0</v>
       </c>
+      <c r="D36" s="11">
+        <v>4100620.0</v>
+      </c>
+      <c r="E36" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F36" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="G36" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="H36" s="11">
         <v>4100578.0</v>
       </c>
@@ -3406,6 +3475,18 @@
       <c r="C48" s="11">
         <v>57.0</v>
       </c>
+      <c r="D48" s="11">
+        <v>4100638.0</v>
+      </c>
+      <c r="E48" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F48" s="11">
+        <v>4.0</v>
+      </c>
+      <c r="G48" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="H48" s="11">
         <v>4100637.0</v>
       </c>
@@ -3494,6 +3575,18 @@
       <c r="C50" s="11">
         <v>60.0</v>
       </c>
+      <c r="D50" s="11">
+        <v>4100620.0</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F50" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="G50" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="H50" s="11">
         <v>4100578.0</v>
       </c>
@@ -3976,7 +4069,7 @@
       <c r="A60" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B60" s="22">
+      <c r="B60" s="21">
         <v>1.0</v>
       </c>
       <c r="C60" s="11">
@@ -4026,7 +4119,7 @@
       <c r="A61" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B61" s="22">
+      <c r="B61" s="21">
         <v>1.0</v>
       </c>
       <c r="C61" s="11">
@@ -4076,7 +4169,7 @@
       <c r="A62" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B62" s="22">
+      <c r="B62" s="21">
         <v>2.0</v>
       </c>
       <c r="C62" s="11">
@@ -4126,7 +4219,7 @@
       <c r="A63" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B63" s="22">
+      <c r="B63" s="21">
         <v>2.0</v>
       </c>
       <c r="C63" s="11">
@@ -4176,7 +4269,7 @@
       <c r="A64" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B64" s="22">
+      <c r="B64" s="21">
         <v>2.0</v>
       </c>
       <c r="C64" s="11">
@@ -4226,7 +4319,7 @@
       <c r="A65" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B65" s="22">
+      <c r="B65" s="21">
         <v>2.0</v>
       </c>
       <c r="C65" s="11">
@@ -4276,7 +4369,7 @@
       <c r="A66" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B66" s="22">
+      <c r="B66" s="21">
         <v>2.0</v>
       </c>
       <c r="C66" s="11">
@@ -4326,7 +4419,7 @@
       <c r="A67" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B67" s="22">
+      <c r="B67" s="21">
         <v>2.0</v>
       </c>
       <c r="C67" s="11">
@@ -4376,7 +4469,7 @@
       <c r="A68" s="5">
         <v>4033.0</v>
       </c>
-      <c r="B68" s="23">
+      <c r="B68" s="22">
         <v>2.0</v>
       </c>
       <c r="C68" s="14">
@@ -4423,10 +4516,10 @@
       <c r="AB68" s="10"/>
     </row>
     <row r="69">
-      <c r="A69" s="24">
+      <c r="A69" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B69" s="25">
+      <c r="B69" s="24">
         <v>1.0</v>
       </c>
       <c r="C69" s="11">
@@ -4473,10 +4566,10 @@
       <c r="AB69" s="10"/>
     </row>
     <row r="70">
-      <c r="A70" s="24">
+      <c r="A70" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B70" s="25">
+      <c r="B70" s="24">
         <v>1.0</v>
       </c>
       <c r="C70" s="11">
@@ -4523,10 +4616,10 @@
       <c r="AB70" s="10"/>
     </row>
     <row r="71">
-      <c r="A71" s="24">
+      <c r="A71" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B71" s="25">
+      <c r="B71" s="24">
         <v>1.0</v>
       </c>
       <c r="C71" s="12">
@@ -4573,10 +4666,10 @@
       <c r="AB71" s="10"/>
     </row>
     <row r="72">
-      <c r="A72" s="24">
+      <c r="A72" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B72" s="25">
+      <c r="B72" s="24">
         <v>1.0</v>
       </c>
       <c r="C72" s="12">
@@ -4623,10 +4716,10 @@
       <c r="AB72" s="10"/>
     </row>
     <row r="73">
-      <c r="A73" s="24">
+      <c r="A73" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B73" s="25">
+      <c r="B73" s="24">
         <v>1.0</v>
       </c>
       <c r="C73" s="12">
@@ -4673,10 +4766,10 @@
       <c r="AB73" s="10"/>
     </row>
     <row r="74">
-      <c r="A74" s="24">
+      <c r="A74" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B74" s="25">
+      <c r="B74" s="24">
         <v>1.0</v>
       </c>
       <c r="C74" s="12">
@@ -4723,10 +4816,10 @@
       <c r="AB74" s="10"/>
     </row>
     <row r="75">
-      <c r="A75" s="24">
+      <c r="A75" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B75" s="25">
+      <c r="B75" s="24">
         <v>1.0</v>
       </c>
       <c r="C75" s="12">
@@ -4773,10 +4866,10 @@
       <c r="AB75" s="10"/>
     </row>
     <row r="76">
-      <c r="A76" s="24">
+      <c r="A76" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B76" s="25">
+      <c r="B76" s="24">
         <v>1.0</v>
       </c>
       <c r="C76" s="12">
@@ -4823,13 +4916,13 @@
       <c r="AB76" s="10"/>
     </row>
     <row r="77">
-      <c r="A77" s="24">
+      <c r="A77" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B77" s="25">
+      <c r="B77" s="24">
         <v>1.0</v>
       </c>
-      <c r="C77" s="25">
+      <c r="C77" s="24">
         <v>96.0</v>
       </c>
       <c r="D77" s="11">
@@ -4873,13 +4966,13 @@
       <c r="AB77" s="10"/>
     </row>
     <row r="78">
-      <c r="A78" s="24">
+      <c r="A78" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B78" s="22">
+      <c r="B78" s="21">
         <v>2.0</v>
       </c>
-      <c r="C78" s="25">
+      <c r="C78" s="24">
         <v>97.0</v>
       </c>
       <c r="D78" s="11">
@@ -4923,13 +5016,13 @@
       <c r="AB78" s="10"/>
     </row>
     <row r="79">
-      <c r="A79" s="24">
+      <c r="A79" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B79" s="22">
+      <c r="B79" s="21">
         <v>2.0</v>
       </c>
-      <c r="C79" s="25">
+      <c r="C79" s="24">
         <v>97.0</v>
       </c>
       <c r="D79" s="11">
@@ -4973,13 +5066,13 @@
       <c r="AB79" s="10"/>
     </row>
     <row r="80">
-      <c r="A80" s="24">
+      <c r="A80" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B80" s="22">
+      <c r="B80" s="21">
         <v>2.0</v>
       </c>
-      <c r="C80" s="25">
+      <c r="C80" s="24">
         <v>97.0</v>
       </c>
       <c r="D80" s="11">
@@ -5023,13 +5116,13 @@
       <c r="AB80" s="10"/>
     </row>
     <row r="81">
-      <c r="A81" s="24">
+      <c r="A81" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B81" s="22">
+      <c r="B81" s="21">
         <v>2.0</v>
       </c>
-      <c r="C81" s="25">
+      <c r="C81" s="24">
         <v>97.0</v>
       </c>
       <c r="D81" s="11">
@@ -5073,13 +5166,13 @@
       <c r="AB81" s="10"/>
     </row>
     <row r="82">
-      <c r="A82" s="24">
+      <c r="A82" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B82" s="22">
+      <c r="B82" s="21">
         <v>2.0</v>
       </c>
-      <c r="C82" s="25">
+      <c r="C82" s="24">
         <v>97.0</v>
       </c>
       <c r="D82" s="11">
@@ -5123,13 +5216,13 @@
       <c r="AB82" s="10"/>
     </row>
     <row r="83">
-      <c r="A83" s="24">
+      <c r="A83" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B83" s="22">
+      <c r="B83" s="21">
         <v>2.0</v>
       </c>
-      <c r="C83" s="25">
+      <c r="C83" s="24">
         <v>97.0</v>
       </c>
       <c r="D83" s="11">
@@ -5173,13 +5266,13 @@
       <c r="AB83" s="10"/>
     </row>
     <row r="84">
-      <c r="A84" s="24">
+      <c r="A84" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B84" s="22">
+      <c r="B84" s="21">
         <v>2.0</v>
       </c>
-      <c r="C84" s="25">
+      <c r="C84" s="24">
         <v>97.0</v>
       </c>
       <c r="D84" s="11">
@@ -5223,13 +5316,13 @@
       <c r="AB84" s="10"/>
     </row>
     <row r="85">
-      <c r="A85" s="24">
+      <c r="A85" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B85" s="22">
+      <c r="B85" s="21">
         <v>2.0</v>
       </c>
-      <c r="C85" s="25">
+      <c r="C85" s="24">
         <v>97.0</v>
       </c>
       <c r="D85" s="11">
@@ -5273,13 +5366,13 @@
       <c r="AB85" s="10"/>
     </row>
     <row r="86">
-      <c r="A86" s="24">
+      <c r="A86" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B86" s="22">
+      <c r="B86" s="21">
         <v>2.0</v>
       </c>
-      <c r="C86" s="25">
+      <c r="C86" s="24">
         <v>97.0</v>
       </c>
       <c r="D86" s="11">
@@ -5323,13 +5416,13 @@
       <c r="AB86" s="10"/>
     </row>
     <row r="87">
-      <c r="A87" s="24">
+      <c r="A87" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B87" s="22">
+      <c r="B87" s="21">
         <v>2.0</v>
       </c>
-      <c r="C87" s="25">
+      <c r="C87" s="24">
         <v>97.0</v>
       </c>
       <c r="D87" s="11">
@@ -5373,13 +5466,13 @@
       <c r="AB87" s="10"/>
     </row>
     <row r="88">
-      <c r="A88" s="24">
+      <c r="A88" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B88" s="22">
+      <c r="B88" s="21">
         <v>2.0</v>
       </c>
-      <c r="C88" s="25">
+      <c r="C88" s="24">
         <v>97.0</v>
       </c>
       <c r="D88" s="11">
@@ -5423,13 +5516,13 @@
       <c r="AB88" s="10"/>
     </row>
     <row r="89">
-      <c r="A89" s="24">
+      <c r="A89" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B89" s="22">
+      <c r="B89" s="21">
         <v>2.0</v>
       </c>
-      <c r="C89" s="25">
+      <c r="C89" s="24">
         <v>97.0</v>
       </c>
       <c r="D89" s="11">
@@ -5473,10 +5566,10 @@
       <c r="AB89" s="10"/>
     </row>
     <row r="90">
-      <c r="A90" s="24">
+      <c r="A90" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B90" s="22">
+      <c r="B90" s="21">
         <v>2.0</v>
       </c>
       <c r="C90" s="12">
@@ -5523,10 +5616,10 @@
       <c r="AB90" s="10"/>
     </row>
     <row r="91">
-      <c r="A91" s="24">
+      <c r="A91" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B91" s="22">
+      <c r="B91" s="21">
         <v>2.0</v>
       </c>
       <c r="C91" s="12">
@@ -5573,10 +5666,10 @@
       <c r="AB91" s="10"/>
     </row>
     <row r="92">
-      <c r="A92" s="24">
+      <c r="A92" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B92" s="22">
+      <c r="B92" s="21">
         <v>2.0</v>
       </c>
       <c r="C92" s="12">
@@ -5623,10 +5716,10 @@
       <c r="AB92" s="10"/>
     </row>
     <row r="93">
-      <c r="A93" s="24">
+      <c r="A93" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B93" s="22">
+      <c r="B93" s="21">
         <v>2.0</v>
       </c>
       <c r="C93" s="12">
@@ -5673,10 +5766,10 @@
       <c r="AB93" s="10"/>
     </row>
     <row r="94">
-      <c r="A94" s="24">
+      <c r="A94" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B94" s="22">
+      <c r="B94" s="21">
         <v>2.0</v>
       </c>
       <c r="C94" s="12">
@@ -5723,10 +5816,10 @@
       <c r="AB94" s="10"/>
     </row>
     <row r="95">
-      <c r="A95" s="24">
+      <c r="A95" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B95" s="22">
+      <c r="B95" s="21">
         <v>2.0</v>
       </c>
       <c r="C95" s="12">
@@ -5773,10 +5866,10 @@
       <c r="AB95" s="10"/>
     </row>
     <row r="96">
-      <c r="A96" s="24">
+      <c r="A96" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B96" s="22">
+      <c r="B96" s="21">
         <v>2.0</v>
       </c>
       <c r="C96" s="12">
@@ -5823,10 +5916,10 @@
       <c r="AB96" s="10"/>
     </row>
     <row r="97">
-      <c r="A97" s="24">
+      <c r="A97" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B97" s="22">
+      <c r="B97" s="21">
         <v>2.0</v>
       </c>
       <c r="C97" s="12">
@@ -5873,10 +5966,10 @@
       <c r="AB97" s="10"/>
     </row>
     <row r="98">
-      <c r="A98" s="24">
+      <c r="A98" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B98" s="22">
+      <c r="B98" s="21">
         <v>2.0</v>
       </c>
       <c r="C98" s="12">
@@ -5923,10 +6016,10 @@
       <c r="AB98" s="10"/>
     </row>
     <row r="99">
-      <c r="A99" s="24">
+      <c r="A99" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B99" s="22">
+      <c r="B99" s="21">
         <v>2.0</v>
       </c>
       <c r="C99" s="12">
@@ -5973,10 +6066,10 @@
       <c r="AB99" s="10"/>
     </row>
     <row r="100">
-      <c r="A100" s="24">
+      <c r="A100" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B100" s="22">
+      <c r="B100" s="21">
         <v>2.0</v>
       </c>
       <c r="C100" s="12">
@@ -6023,10 +6116,10 @@
       <c r="AB100" s="10"/>
     </row>
     <row r="101">
-      <c r="A101" s="24">
+      <c r="A101" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B101" s="22">
+      <c r="B101" s="21">
         <v>2.0</v>
       </c>
       <c r="C101" s="12">
@@ -6073,10 +6166,10 @@
       <c r="AB101" s="10"/>
     </row>
     <row r="102">
-      <c r="A102" s="24">
+      <c r="A102" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B102" s="22">
+      <c r="B102" s="21">
         <v>2.0</v>
       </c>
       <c r="C102" s="12">
@@ -6123,10 +6216,10 @@
       <c r="AB102" s="10"/>
     </row>
     <row r="103">
-      <c r="A103" s="24">
+      <c r="A103" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B103" s="22">
+      <c r="B103" s="21">
         <v>2.0</v>
       </c>
       <c r="C103" s="12">
@@ -6173,10 +6266,10 @@
       <c r="AB103" s="10"/>
     </row>
     <row r="104">
-      <c r="A104" s="24">
+      <c r="A104" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B104" s="22">
+      <c r="B104" s="21">
         <v>2.0</v>
       </c>
       <c r="C104" s="12">
@@ -6223,10 +6316,10 @@
       <c r="AB104" s="10"/>
     </row>
     <row r="105">
-      <c r="A105" s="24">
+      <c r="A105" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B105" s="22">
+      <c r="B105" s="21">
         <v>2.0</v>
       </c>
       <c r="C105" s="12">
@@ -6273,10 +6366,10 @@
       <c r="AB105" s="10"/>
     </row>
     <row r="106">
-      <c r="A106" s="24">
+      <c r="A106" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B106" s="22">
+      <c r="B106" s="21">
         <v>2.0</v>
       </c>
       <c r="C106" s="12">
@@ -6323,10 +6416,10 @@
       <c r="AB106" s="10"/>
     </row>
     <row r="107">
-      <c r="A107" s="24">
+      <c r="A107" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B107" s="22">
+      <c r="B107" s="21">
         <v>2.0</v>
       </c>
       <c r="C107" s="12">
@@ -6373,10 +6466,10 @@
       <c r="AB107" s="10"/>
     </row>
     <row r="108">
-      <c r="A108" s="24">
+      <c r="A108" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B108" s="22">
+      <c r="B108" s="21">
         <v>2.0</v>
       </c>
       <c r="C108" s="12">
@@ -6423,10 +6516,10 @@
       <c r="AB108" s="10"/>
     </row>
     <row r="109">
-      <c r="A109" s="24">
+      <c r="A109" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B109" s="22">
+      <c r="B109" s="21">
         <v>2.0</v>
       </c>
       <c r="C109" s="12">
@@ -6473,10 +6566,10 @@
       <c r="AB109" s="10"/>
     </row>
     <row r="110">
-      <c r="A110" s="24">
+      <c r="A110" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B110" s="22">
+      <c r="B110" s="21">
         <v>2.0</v>
       </c>
       <c r="C110" s="12">
@@ -6523,10 +6616,10 @@
       <c r="AB110" s="10"/>
     </row>
     <row r="111">
-      <c r="A111" s="24">
+      <c r="A111" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B111" s="22">
+      <c r="B111" s="21">
         <v>2.0</v>
       </c>
       <c r="C111" s="12">
@@ -6573,10 +6666,10 @@
       <c r="AB111" s="10"/>
     </row>
     <row r="112">
-      <c r="A112" s="24">
+      <c r="A112" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B112" s="22">
+      <c r="B112" s="21">
         <v>2.0</v>
       </c>
       <c r="C112" s="12">
@@ -6623,10 +6716,10 @@
       <c r="AB112" s="10"/>
     </row>
     <row r="113">
-      <c r="A113" s="24">
+      <c r="A113" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B113" s="22">
+      <c r="B113" s="21">
         <v>2.0</v>
       </c>
       <c r="C113" s="12">
@@ -6673,10 +6766,10 @@
       <c r="AB113" s="10"/>
     </row>
     <row r="114">
-      <c r="A114" s="24">
+      <c r="A114" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B114" s="22">
+      <c r="B114" s="21">
         <v>2.0</v>
       </c>
       <c r="C114" s="12">
@@ -6723,10 +6816,10 @@
       <c r="AB114" s="10"/>
     </row>
     <row r="115">
-      <c r="A115" s="24">
+      <c r="A115" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B115" s="22">
+      <c r="B115" s="21">
         <v>2.0</v>
       </c>
       <c r="C115" s="12">
@@ -6773,10 +6866,10 @@
       <c r="AB115" s="10"/>
     </row>
     <row r="116">
-      <c r="A116" s="24">
+      <c r="A116" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B116" s="22">
+      <c r="B116" s="21">
         <v>2.0</v>
       </c>
       <c r="C116" s="12">
@@ -6823,10 +6916,10 @@
       <c r="AB116" s="10"/>
     </row>
     <row r="117">
-      <c r="A117" s="24">
+      <c r="A117" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B117" s="22">
+      <c r="B117" s="21">
         <v>2.0</v>
       </c>
       <c r="C117" s="12">
@@ -6873,10 +6966,10 @@
       <c r="AB117" s="10"/>
     </row>
     <row r="118">
-      <c r="A118" s="24">
+      <c r="A118" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B118" s="22">
+      <c r="B118" s="21">
         <v>2.0</v>
       </c>
       <c r="C118" s="12">
@@ -6923,10 +7016,10 @@
       <c r="AB118" s="10"/>
     </row>
     <row r="119">
-      <c r="A119" s="24">
+      <c r="A119" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B119" s="22">
+      <c r="B119" s="21">
         <v>2.0</v>
       </c>
       <c r="C119" s="12">
@@ -6973,10 +7066,10 @@
       <c r="AB119" s="10"/>
     </row>
     <row r="120">
-      <c r="A120" s="24">
+      <c r="A120" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B120" s="22">
+      <c r="B120" s="21">
         <v>2.0</v>
       </c>
       <c r="C120" s="12">
@@ -7023,10 +7116,10 @@
       <c r="AB120" s="10"/>
     </row>
     <row r="121">
-      <c r="A121" s="24">
+      <c r="A121" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B121" s="22">
+      <c r="B121" s="21">
         <v>2.0</v>
       </c>
       <c r="C121" s="12">
@@ -7073,10 +7166,10 @@
       <c r="AB121" s="10"/>
     </row>
     <row r="122">
-      <c r="A122" s="24">
+      <c r="A122" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B122" s="22">
+      <c r="B122" s="21">
         <v>2.0</v>
       </c>
       <c r="C122" s="12">
@@ -7123,10 +7216,10 @@
       <c r="AB122" s="10"/>
     </row>
     <row r="123">
-      <c r="A123" s="24">
+      <c r="A123" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B123" s="22">
+      <c r="B123" s="21">
         <v>2.0</v>
       </c>
       <c r="C123" s="12">
@@ -7173,10 +7266,10 @@
       <c r="AB123" s="10"/>
     </row>
     <row r="124">
-      <c r="A124" s="24">
+      <c r="A124" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B124" s="22">
+      <c r="B124" s="21">
         <v>2.0</v>
       </c>
       <c r="C124" s="12">
@@ -7223,10 +7316,10 @@
       <c r="AB124" s="10"/>
     </row>
     <row r="125">
-      <c r="A125" s="24">
+      <c r="A125" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B125" s="22">
+      <c r="B125" s="21">
         <v>2.0</v>
       </c>
       <c r="C125" s="12">
@@ -7273,10 +7366,10 @@
       <c r="AB125" s="10"/>
     </row>
     <row r="126">
-      <c r="A126" s="24">
+      <c r="A126" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B126" s="22">
+      <c r="B126" s="21">
         <v>2.0</v>
       </c>
       <c r="C126" s="12">
@@ -7323,10 +7416,10 @@
       <c r="AB126" s="10"/>
     </row>
     <row r="127">
-      <c r="A127" s="24">
+      <c r="A127" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B127" s="22">
+      <c r="B127" s="21">
         <v>2.0</v>
       </c>
       <c r="C127" s="12">
@@ -7373,10 +7466,10 @@
       <c r="AB127" s="10"/>
     </row>
     <row r="128">
-      <c r="A128" s="24">
+      <c r="A128" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B128" s="22">
+      <c r="B128" s="21">
         <v>2.0</v>
       </c>
       <c r="C128" s="12">
@@ -7423,10 +7516,10 @@
       <c r="AB128" s="10"/>
     </row>
     <row r="129">
-      <c r="A129" s="24">
+      <c r="A129" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B129" s="22">
+      <c r="B129" s="21">
         <v>2.0</v>
       </c>
       <c r="C129" s="12">
@@ -7473,10 +7566,10 @@
       <c r="AB129" s="10"/>
     </row>
     <row r="130">
-      <c r="A130" s="24">
+      <c r="A130" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B130" s="22">
+      <c r="B130" s="21">
         <v>2.0</v>
       </c>
       <c r="C130" s="12">
@@ -7523,10 +7616,10 @@
       <c r="AB130" s="10"/>
     </row>
     <row r="131">
-      <c r="A131" s="24">
+      <c r="A131" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B131" s="22">
+      <c r="B131" s="21">
         <v>2.0</v>
       </c>
       <c r="C131" s="12">
@@ -7573,10 +7666,10 @@
       <c r="AB131" s="10"/>
     </row>
     <row r="132">
-      <c r="A132" s="24">
+      <c r="A132" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B132" s="22">
+      <c r="B132" s="21">
         <v>2.0</v>
       </c>
       <c r="C132" s="12">
@@ -7623,10 +7716,10 @@
       <c r="AB132" s="10"/>
     </row>
     <row r="133">
-      <c r="A133" s="24">
+      <c r="A133" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B133" s="22">
+      <c r="B133" s="21">
         <v>2.0</v>
       </c>
       <c r="C133" s="12">
@@ -7673,10 +7766,10 @@
       <c r="AB133" s="10"/>
     </row>
     <row r="134">
-      <c r="A134" s="24">
+      <c r="A134" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B134" s="22">
+      <c r="B134" s="21">
         <v>2.0</v>
       </c>
       <c r="C134" s="12">
@@ -7723,10 +7816,10 @@
       <c r="AB134" s="10"/>
     </row>
     <row r="135">
-      <c r="A135" s="24">
+      <c r="A135" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B135" s="22">
+      <c r="B135" s="21">
         <v>2.0</v>
       </c>
       <c r="C135" s="12">
@@ -7773,10 +7866,10 @@
       <c r="AB135" s="10"/>
     </row>
     <row r="136">
-      <c r="A136" s="24">
+      <c r="A136" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B136" s="22">
+      <c r="B136" s="21">
         <v>2.0</v>
       </c>
       <c r="C136" s="12">
@@ -7823,10 +7916,10 @@
       <c r="AB136" s="10"/>
     </row>
     <row r="137">
-      <c r="A137" s="24">
+      <c r="A137" s="23">
         <v>4028.0</v>
       </c>
-      <c r="B137" s="23">
+      <c r="B137" s="22">
         <v>2.0</v>
       </c>
       <c r="C137" s="15">
@@ -7873,10 +7966,10 @@
       <c r="AB137" s="10"/>
     </row>
     <row r="138">
-      <c r="A138" s="24">
+      <c r="A138" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B138" s="22">
+      <c r="B138" s="21">
         <v>2.0</v>
       </c>
       <c r="C138" s="12">
@@ -7923,10 +8016,10 @@
       <c r="AB138" s="10"/>
     </row>
     <row r="139">
-      <c r="A139" s="24">
+      <c r="A139" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B139" s="22">
+      <c r="B139" s="21">
         <v>2.0</v>
       </c>
       <c r="C139" s="12">
@@ -7973,10 +8066,10 @@
       <c r="AB139" s="10"/>
     </row>
     <row r="140">
-      <c r="A140" s="24">
+      <c r="A140" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B140" s="22">
+      <c r="B140" s="21">
         <v>2.0</v>
       </c>
       <c r="C140" s="12">
@@ -8023,10 +8116,10 @@
       <c r="AB140" s="10"/>
     </row>
     <row r="141">
-      <c r="A141" s="24">
+      <c r="A141" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B141" s="22">
+      <c r="B141" s="21">
         <v>2.0</v>
       </c>
       <c r="C141" s="12">
@@ -8073,10 +8166,10 @@
       <c r="AB141" s="10"/>
     </row>
     <row r="142">
-      <c r="A142" s="24">
+      <c r="A142" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B142" s="22">
+      <c r="B142" s="21">
         <v>2.0</v>
       </c>
       <c r="C142" s="12">
@@ -8123,10 +8216,10 @@
       <c r="AB142" s="10"/>
     </row>
     <row r="143">
-      <c r="A143" s="24">
+      <c r="A143" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B143" s="22">
+      <c r="B143" s="21">
         <v>2.0</v>
       </c>
       <c r="C143" s="12">
@@ -8173,10 +8266,10 @@
       <c r="AB143" s="10"/>
     </row>
     <row r="144">
-      <c r="A144" s="24">
+      <c r="A144" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B144" s="22">
+      <c r="B144" s="21">
         <v>2.0</v>
       </c>
       <c r="C144" s="12">
@@ -8223,10 +8316,10 @@
       <c r="AB144" s="10"/>
     </row>
     <row r="145">
-      <c r="A145" s="24">
+      <c r="A145" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B145" s="22">
+      <c r="B145" s="21">
         <v>2.0</v>
       </c>
       <c r="C145" s="12">
@@ -8273,10 +8366,10 @@
       <c r="AB145" s="10"/>
     </row>
     <row r="146">
-      <c r="A146" s="24">
+      <c r="A146" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B146" s="22">
+      <c r="B146" s="21">
         <v>2.0</v>
       </c>
       <c r="C146" s="12">
@@ -8323,10 +8416,10 @@
       <c r="AB146" s="10"/>
     </row>
     <row r="147">
-      <c r="A147" s="24">
+      <c r="A147" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B147" s="22">
+      <c r="B147" s="21">
         <v>2.0</v>
       </c>
       <c r="C147" s="12">
@@ -8373,10 +8466,10 @@
       <c r="AB147" s="10"/>
     </row>
     <row r="148">
-      <c r="A148" s="24">
+      <c r="A148" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B148" s="22">
+      <c r="B148" s="21">
         <v>2.0</v>
       </c>
       <c r="C148" s="12">
@@ -8423,10 +8516,10 @@
       <c r="AB148" s="10"/>
     </row>
     <row r="149">
-      <c r="A149" s="24">
+      <c r="A149" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B149" s="22">
+      <c r="B149" s="21">
         <v>2.0</v>
       </c>
       <c r="C149" s="12">
@@ -8473,10 +8566,10 @@
       <c r="AB149" s="10"/>
     </row>
     <row r="150">
-      <c r="A150" s="24">
+      <c r="A150" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B150" s="22">
+      <c r="B150" s="21">
         <v>2.0</v>
       </c>
       <c r="C150" s="12">
@@ -8523,10 +8616,10 @@
       <c r="AB150" s="10"/>
     </row>
     <row r="151">
-      <c r="A151" s="24">
+      <c r="A151" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B151" s="22">
+      <c r="B151" s="21">
         <v>2.0</v>
       </c>
       <c r="C151" s="12">
@@ -8573,10 +8666,10 @@
       <c r="AB151" s="10"/>
     </row>
     <row r="152">
-      <c r="A152" s="24">
+      <c r="A152" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B152" s="22">
+      <c r="B152" s="21">
         <v>2.0</v>
       </c>
       <c r="C152" s="12">
@@ -8623,10 +8716,10 @@
       <c r="AB152" s="10"/>
     </row>
     <row r="153">
-      <c r="A153" s="24">
+      <c r="A153" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B153" s="22">
+      <c r="B153" s="21">
         <v>2.0</v>
       </c>
       <c r="C153" s="12">
@@ -8673,10 +8766,10 @@
       <c r="AB153" s="10"/>
     </row>
     <row r="154">
-      <c r="A154" s="24">
+      <c r="A154" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B154" s="22">
+      <c r="B154" s="21">
         <v>2.0</v>
       </c>
       <c r="C154" s="12">
@@ -8723,10 +8816,10 @@
       <c r="AB154" s="10"/>
     </row>
     <row r="155">
-      <c r="A155" s="24">
+      <c r="A155" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B155" s="22">
+      <c r="B155" s="21">
         <v>2.0</v>
       </c>
       <c r="C155" s="12">
@@ -8773,10 +8866,10 @@
       <c r="AB155" s="10"/>
     </row>
     <row r="156">
-      <c r="A156" s="24">
+      <c r="A156" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B156" s="22">
+      <c r="B156" s="21">
         <v>2.0</v>
       </c>
       <c r="C156" s="12">
@@ -8823,10 +8916,10 @@
       <c r="AB156" s="10"/>
     </row>
     <row r="157">
-      <c r="A157" s="24">
+      <c r="A157" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B157" s="22">
+      <c r="B157" s="21">
         <v>2.0</v>
       </c>
       <c r="C157" s="12">
@@ -8873,10 +8966,10 @@
       <c r="AB157" s="10"/>
     </row>
     <row r="158">
-      <c r="A158" s="24">
+      <c r="A158" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B158" s="22">
+      <c r="B158" s="21">
         <v>2.0</v>
       </c>
       <c r="C158" s="12">
@@ -8923,10 +9016,10 @@
       <c r="AB158" s="10"/>
     </row>
     <row r="159">
-      <c r="A159" s="24">
+      <c r="A159" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B159" s="22">
+      <c r="B159" s="21">
         <v>2.0</v>
       </c>
       <c r="C159" s="12">
@@ -8973,10 +9066,10 @@
       <c r="AB159" s="10"/>
     </row>
     <row r="160">
-      <c r="A160" s="24">
+      <c r="A160" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B160" s="22">
+      <c r="B160" s="21">
         <v>2.0</v>
       </c>
       <c r="C160" s="12">
@@ -9023,10 +9116,10 @@
       <c r="AB160" s="10"/>
     </row>
     <row r="161">
-      <c r="A161" s="24">
+      <c r="A161" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B161" s="22">
+      <c r="B161" s="21">
         <v>2.0</v>
       </c>
       <c r="C161" s="12">
@@ -9073,10 +9166,10 @@
       <c r="AB161" s="10"/>
     </row>
     <row r="162">
-      <c r="A162" s="24">
+      <c r="A162" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B162" s="22">
+      <c r="B162" s="21">
         <v>2.0</v>
       </c>
       <c r="C162" s="12">
@@ -9123,10 +9216,10 @@
       <c r="AB162" s="10"/>
     </row>
     <row r="163">
-      <c r="A163" s="24">
+      <c r="A163" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B163" s="22">
+      <c r="B163" s="21">
         <v>2.0</v>
       </c>
       <c r="C163" s="12">
@@ -9173,10 +9266,10 @@
       <c r="AB163" s="10"/>
     </row>
     <row r="164">
-      <c r="A164" s="24">
+      <c r="A164" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B164" s="22">
+      <c r="B164" s="21">
         <v>2.0</v>
       </c>
       <c r="C164" s="12">
@@ -9223,10 +9316,10 @@
       <c r="AB164" s="10"/>
     </row>
     <row r="165">
-      <c r="A165" s="24">
+      <c r="A165" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B165" s="22">
+      <c r="B165" s="21">
         <v>2.0</v>
       </c>
       <c r="C165" s="12">
@@ -9273,10 +9366,10 @@
       <c r="AB165" s="10"/>
     </row>
     <row r="166">
-      <c r="A166" s="24">
+      <c r="A166" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B166" s="22">
+      <c r="B166" s="21">
         <v>2.0</v>
       </c>
       <c r="C166" s="12">
@@ -9323,10 +9416,10 @@
       <c r="AB166" s="10"/>
     </row>
     <row r="167">
-      <c r="A167" s="24">
+      <c r="A167" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B167" s="22">
+      <c r="B167" s="21">
         <v>2.0</v>
       </c>
       <c r="C167" s="12">
@@ -9373,10 +9466,10 @@
       <c r="AB167" s="10"/>
     </row>
     <row r="168">
-      <c r="A168" s="24">
+      <c r="A168" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B168" s="22">
+      <c r="B168" s="21">
         <v>2.0</v>
       </c>
       <c r="C168" s="12">
@@ -9423,10 +9516,10 @@
       <c r="AB168" s="10"/>
     </row>
     <row r="169">
-      <c r="A169" s="24">
+      <c r="A169" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B169" s="22">
+      <c r="B169" s="21">
         <v>2.0</v>
       </c>
       <c r="C169" s="12">
@@ -9473,10 +9566,10 @@
       <c r="AB169" s="10"/>
     </row>
     <row r="170">
-      <c r="A170" s="24">
+      <c r="A170" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B170" s="22">
+      <c r="B170" s="21">
         <v>2.0</v>
       </c>
       <c r="C170" s="12">
@@ -9523,10 +9616,10 @@
       <c r="AB170" s="10"/>
     </row>
     <row r="171">
-      <c r="A171" s="24">
+      <c r="A171" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B171" s="22">
+      <c r="B171" s="21">
         <v>2.0</v>
       </c>
       <c r="C171" s="12">
@@ -9573,10 +9666,10 @@
       <c r="AB171" s="10"/>
     </row>
     <row r="172">
-      <c r="A172" s="24">
+      <c r="A172" s="23">
         <v>4032.0</v>
       </c>
-      <c r="B172" s="23">
+      <c r="B172" s="22">
         <v>2.0</v>
       </c>
       <c r="C172" s="15">
@@ -9623,10 +9716,10 @@
       <c r="AB172" s="10"/>
     </row>
     <row r="173">
-      <c r="A173" s="24">
+      <c r="A173" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B173" s="22">
+      <c r="B173" s="21">
         <v>1.0</v>
       </c>
       <c r="C173" s="12">
@@ -9673,10 +9766,10 @@
       <c r="AB173" s="10"/>
     </row>
     <row r="174">
-      <c r="A174" s="24">
+      <c r="A174" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B174" s="22">
+      <c r="B174" s="21">
         <v>1.0</v>
       </c>
       <c r="C174" s="12">
@@ -9723,10 +9816,10 @@
       <c r="AB174" s="10"/>
     </row>
     <row r="175">
-      <c r="A175" s="24">
+      <c r="A175" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B175" s="22">
+      <c r="B175" s="21">
         <v>1.0</v>
       </c>
       <c r="C175" s="12">
@@ -9773,10 +9866,10 @@
       <c r="AB175" s="10"/>
     </row>
     <row r="176">
-      <c r="A176" s="24">
+      <c r="A176" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B176" s="22">
+      <c r="B176" s="21">
         <v>1.0</v>
       </c>
       <c r="C176" s="12">
@@ -9823,10 +9916,10 @@
       <c r="AB176" s="10"/>
     </row>
     <row r="177">
-      <c r="A177" s="24">
+      <c r="A177" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B177" s="22">
+      <c r="B177" s="21">
         <v>1.0</v>
       </c>
       <c r="C177" s="12">
@@ -9873,10 +9966,10 @@
       <c r="AB177" s="10"/>
     </row>
     <row r="178">
-      <c r="A178" s="24">
+      <c r="A178" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B178" s="22">
+      <c r="B178" s="21">
         <v>1.0</v>
       </c>
       <c r="C178" s="12">
@@ -9923,10 +10016,10 @@
       <c r="AB178" s="10"/>
     </row>
     <row r="179">
-      <c r="A179" s="24">
+      <c r="A179" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B179" s="22">
+      <c r="B179" s="21">
         <v>1.0</v>
       </c>
       <c r="C179" s="12">
@@ -9973,10 +10066,10 @@
       <c r="AB179" s="10"/>
     </row>
     <row r="180">
-      <c r="A180" s="24">
+      <c r="A180" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B180" s="22">
+      <c r="B180" s="21">
         <v>1.0</v>
       </c>
       <c r="C180" s="12">
@@ -10023,10 +10116,10 @@
       <c r="AB180" s="10"/>
     </row>
     <row r="181">
-      <c r="A181" s="24">
+      <c r="A181" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B181" s="22">
+      <c r="B181" s="21">
         <v>1.0</v>
       </c>
       <c r="C181" s="12">
@@ -10073,10 +10166,10 @@
       <c r="AB181" s="10"/>
     </row>
     <row r="182">
-      <c r="A182" s="24">
+      <c r="A182" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B182" s="22">
+      <c r="B182" s="21">
         <v>1.0</v>
       </c>
       <c r="C182" s="12">
@@ -10123,10 +10216,10 @@
       <c r="AB182" s="10"/>
     </row>
     <row r="183">
-      <c r="A183" s="24">
+      <c r="A183" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B183" s="22">
+      <c r="B183" s="21">
         <v>1.0</v>
       </c>
       <c r="C183" s="12">
@@ -10173,10 +10266,10 @@
       <c r="AB183" s="10"/>
     </row>
     <row r="184">
-      <c r="A184" s="24">
+      <c r="A184" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B184" s="22">
+      <c r="B184" s="21">
         <v>1.0</v>
       </c>
       <c r="C184" s="12">
@@ -10223,10 +10316,10 @@
       <c r="AB184" s="10"/>
     </row>
     <row r="185">
-      <c r="A185" s="24">
+      <c r="A185" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B185" s="22">
+      <c r="B185" s="21">
         <v>1.0</v>
       </c>
       <c r="C185" s="12">
@@ -10244,7 +10337,7 @@
       <c r="G185" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H185" s="26">
+      <c r="H185" s="25">
         <v>4201258.0</v>
       </c>
       <c r="I185" s="11"/>
@@ -10271,10 +10364,10 @@
       <c r="AB185" s="10"/>
     </row>
     <row r="186">
-      <c r="A186" s="24">
+      <c r="A186" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B186" s="22">
+      <c r="B186" s="21">
         <v>2.0</v>
       </c>
       <c r="C186" s="12">
@@ -10321,10 +10414,10 @@
       <c r="AB186" s="10"/>
     </row>
     <row r="187">
-      <c r="A187" s="24">
+      <c r="A187" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B187" s="22">
+      <c r="B187" s="21">
         <v>2.0</v>
       </c>
       <c r="C187" s="12">
@@ -10371,10 +10464,10 @@
       <c r="AB187" s="10"/>
     </row>
     <row r="188">
-      <c r="A188" s="24">
+      <c r="A188" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B188" s="22">
+      <c r="B188" s="21">
         <v>2.0</v>
       </c>
       <c r="C188" s="12">
@@ -10421,10 +10514,10 @@
       <c r="AB188" s="10"/>
     </row>
     <row r="189">
-      <c r="A189" s="24">
+      <c r="A189" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B189" s="22">
+      <c r="B189" s="21">
         <v>2.0</v>
       </c>
       <c r="C189" s="12">
@@ -10471,10 +10564,10 @@
       <c r="AB189" s="10"/>
     </row>
     <row r="190">
-      <c r="A190" s="24">
+      <c r="A190" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B190" s="22">
+      <c r="B190" s="21">
         <v>2.0</v>
       </c>
       <c r="C190" s="12">
@@ -10521,10 +10614,10 @@
       <c r="AB190" s="10"/>
     </row>
     <row r="191">
-      <c r="A191" s="24">
+      <c r="A191" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B191" s="22">
+      <c r="B191" s="21">
         <v>2.0</v>
       </c>
       <c r="C191" s="12">
@@ -10571,10 +10664,10 @@
       <c r="AB191" s="10"/>
     </row>
     <row r="192">
-      <c r="A192" s="24">
+      <c r="A192" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B192" s="22">
+      <c r="B192" s="21">
         <v>2.0</v>
       </c>
       <c r="C192" s="12">
@@ -10621,10 +10714,10 @@
       <c r="AB192" s="10"/>
     </row>
     <row r="193">
-      <c r="A193" s="24">
+      <c r="A193" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B193" s="22">
+      <c r="B193" s="21">
         <v>2.0</v>
       </c>
       <c r="C193" s="12">
@@ -10642,11 +10735,11 @@
       <c r="G193" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H193" s="26">
+      <c r="H193" s="25">
         <v>4100804.0</v>
       </c>
-      <c r="I193" s="26"/>
-      <c r="J193" s="27"/>
+      <c r="I193" s="25"/>
+      <c r="J193" s="26"/>
       <c r="K193" s="10"/>
       <c r="L193" s="10"/>
       <c r="M193" s="10"/>
@@ -10667,10 +10760,10 @@
       <c r="AB193" s="10"/>
     </row>
     <row r="194">
-      <c r="A194" s="24">
+      <c r="A194" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B194" s="22">
+      <c r="B194" s="21">
         <v>2.0</v>
       </c>
       <c r="C194" s="12">
@@ -10717,10 +10810,10 @@
       <c r="AB194" s="10"/>
     </row>
     <row r="195">
-      <c r="A195" s="24">
+      <c r="A195" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B195" s="22">
+      <c r="B195" s="21">
         <v>2.0</v>
       </c>
       <c r="C195" s="12">
@@ -10767,10 +10860,10 @@
       <c r="AB195" s="10"/>
     </row>
     <row r="196">
-      <c r="A196" s="24">
+      <c r="A196" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B196" s="22">
+      <c r="B196" s="21">
         <v>2.0</v>
       </c>
       <c r="C196" s="12">
@@ -10817,10 +10910,10 @@
       <c r="AB196" s="10"/>
     </row>
     <row r="197">
-      <c r="A197" s="24">
+      <c r="A197" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B197" s="22">
+      <c r="B197" s="21">
         <v>2.0</v>
       </c>
       <c r="C197" s="12">
@@ -10867,10 +10960,10 @@
       <c r="AB197" s="10"/>
     </row>
     <row r="198">
-      <c r="A198" s="24">
+      <c r="A198" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B198" s="22">
+      <c r="B198" s="21">
         <v>2.0</v>
       </c>
       <c r="C198" s="12">
@@ -10917,10 +11010,10 @@
       <c r="AB198" s="10"/>
     </row>
     <row r="199">
-      <c r="A199" s="24">
+      <c r="A199" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B199" s="22">
+      <c r="B199" s="21">
         <v>2.0</v>
       </c>
       <c r="C199" s="12">
@@ -10938,11 +11031,11 @@
       <c r="G199" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H199" s="26">
+      <c r="H199" s="25">
         <v>4100582.0</v>
       </c>
-      <c r="I199" s="26"/>
-      <c r="J199" s="27" t="s">
+      <c r="I199" s="25"/>
+      <c r="J199" s="26" t="s">
         <v>13</v>
       </c>
       <c r="K199" s="10"/>
@@ -10965,10 +11058,10 @@
       <c r="AB199" s="10"/>
     </row>
     <row r="200">
-      <c r="A200" s="24">
+      <c r="A200" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B200" s="22">
+      <c r="B200" s="21">
         <v>2.0</v>
       </c>
       <c r="C200" s="12">
@@ -11015,10 +11108,10 @@
       <c r="AB200" s="10"/>
     </row>
     <row r="201">
-      <c r="A201" s="24">
+      <c r="A201" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B201" s="22">
+      <c r="B201" s="21">
         <v>2.0</v>
       </c>
       <c r="C201" s="12">
@@ -11065,10 +11158,10 @@
       <c r="AB201" s="10"/>
     </row>
     <row r="202">
-      <c r="A202" s="24">
+      <c r="A202" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B202" s="22">
+      <c r="B202" s="21">
         <v>2.0</v>
       </c>
       <c r="C202" s="12">
@@ -11115,10 +11208,10 @@
       <c r="AB202" s="10"/>
     </row>
     <row r="203">
-      <c r="A203" s="24">
+      <c r="A203" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B203" s="22">
+      <c r="B203" s="21">
         <v>2.0</v>
       </c>
       <c r="C203" s="12">
@@ -11165,10 +11258,10 @@
       <c r="AB203" s="10"/>
     </row>
     <row r="204">
-      <c r="A204" s="24">
+      <c r="A204" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B204" s="22">
+      <c r="B204" s="21">
         <v>2.0</v>
       </c>
       <c r="C204" s="12">
@@ -11215,10 +11308,10 @@
       <c r="AB204" s="10"/>
     </row>
     <row r="205">
-      <c r="A205" s="24">
+      <c r="A205" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B205" s="22">
+      <c r="B205" s="21">
         <v>2.0</v>
       </c>
       <c r="C205" s="12">
@@ -11265,10 +11358,10 @@
       <c r="AB205" s="10"/>
     </row>
     <row r="206">
-      <c r="A206" s="24">
+      <c r="A206" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B206" s="22">
+      <c r="B206" s="21">
         <v>2.0</v>
       </c>
       <c r="C206" s="12">
@@ -11315,10 +11408,10 @@
       <c r="AB206" s="10"/>
     </row>
     <row r="207">
-      <c r="A207" s="24">
+      <c r="A207" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B207" s="22">
+      <c r="B207" s="21">
         <v>2.0</v>
       </c>
       <c r="C207" s="12">
@@ -11365,10 +11458,10 @@
       <c r="AB207" s="10"/>
     </row>
     <row r="208">
-      <c r="A208" s="24">
+      <c r="A208" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B208" s="22">
+      <c r="B208" s="21">
         <v>2.0</v>
       </c>
       <c r="C208" s="12">
@@ -11415,10 +11508,10 @@
       <c r="AB208" s="10"/>
     </row>
     <row r="209">
-      <c r="A209" s="24">
+      <c r="A209" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B209" s="22">
+      <c r="B209" s="21">
         <v>2.0</v>
       </c>
       <c r="C209" s="12">
@@ -11465,10 +11558,10 @@
       <c r="AB209" s="10"/>
     </row>
     <row r="210">
-      <c r="A210" s="24">
+      <c r="A210" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B210" s="22">
+      <c r="B210" s="21">
         <v>2.0</v>
       </c>
       <c r="C210" s="12">
@@ -11515,10 +11608,10 @@
       <c r="AB210" s="10"/>
     </row>
     <row r="211">
-      <c r="A211" s="24">
+      <c r="A211" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B211" s="22">
+      <c r="B211" s="21">
         <v>2.0</v>
       </c>
       <c r="C211" s="12">
@@ -11565,10 +11658,10 @@
       <c r="AB211" s="10"/>
     </row>
     <row r="212">
-      <c r="A212" s="24">
+      <c r="A212" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B212" s="22">
+      <c r="B212" s="21">
         <v>2.0</v>
       </c>
       <c r="C212" s="12">
@@ -11615,10 +11708,10 @@
       <c r="AB212" s="10"/>
     </row>
     <row r="213">
-      <c r="A213" s="24">
+      <c r="A213" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B213" s="22">
+      <c r="B213" s="21">
         <v>2.0</v>
       </c>
       <c r="C213" s="12">
@@ -11665,10 +11758,10 @@
       <c r="AB213" s="10"/>
     </row>
     <row r="214">
-      <c r="A214" s="24">
+      <c r="A214" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B214" s="22">
+      <c r="B214" s="21">
         <v>2.0</v>
       </c>
       <c r="C214" s="12">
@@ -11715,10 +11808,10 @@
       <c r="AB214" s="10"/>
     </row>
     <row r="215">
-      <c r="A215" s="24">
+      <c r="A215" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B215" s="22">
+      <c r="B215" s="21">
         <v>2.0</v>
       </c>
       <c r="C215" s="12">
@@ -11765,10 +11858,10 @@
       <c r="AB215" s="10"/>
     </row>
     <row r="216">
-      <c r="A216" s="24">
+      <c r="A216" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B216" s="22">
+      <c r="B216" s="21">
         <v>2.0</v>
       </c>
       <c r="C216" s="12">
@@ -11815,10 +11908,10 @@
       <c r="AB216" s="10"/>
     </row>
     <row r="217">
-      <c r="A217" s="24">
+      <c r="A217" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B217" s="22">
+      <c r="B217" s="21">
         <v>2.0</v>
       </c>
       <c r="C217" s="12">
@@ -11865,10 +11958,10 @@
       <c r="AB217" s="10"/>
     </row>
     <row r="218">
-      <c r="A218" s="24">
+      <c r="A218" s="23">
         <v>4034.0</v>
       </c>
-      <c r="B218" s="23">
+      <c r="B218" s="22">
         <v>2.0</v>
       </c>
       <c r="C218" s="15">
@@ -35225,32 +35318,6 @@
       <c r="AB995" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="G47:G48"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="G49:G50"/>
-  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>